<commit_message>
Restore 28 student 955 Academic Support requests to T2
T2 V3 removed all 955 requests along with 849/851/830. Theology was
restored earlier but 955 was missed. JC confirmed all 28 from SIS.

T2 final: 6,556 rows (6,552 unique), 804 students, 144 courses, 28×955.

Credit Audit updated (period slot methodology):
- 0 over cap
- 757 at 35 credits (full schedule)
- 28 full schedule via credit-exempt course (955 = 0cr, 1 slot)
- 19 under-scheduled (down from 47)

All Students Schedule Status regenerated with updated counts.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/All_Students_Schedule_Status_2026_27.xlsx
+++ b/All_Students_Schedule_Status_2026_27.xlsx
@@ -21,7 +21,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -39,6 +39,12 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="00008000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="000000FF"/>
       <sz val="10"/>
     </font>
     <font>
@@ -84,7 +90,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
@@ -97,6 +103,8 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -470,7 +478,7 @@
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="23" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -2414,15 +2422,15 @@
         <v>30</v>
       </c>
       <c r="E67" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F67" s="8" t="inlineStr">
         <is>
-          <t>INCOMPLETE</t>
+          <t>FULL (Credit-Exempt)</t>
         </is>
       </c>
       <c r="G67" s="5" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="68">
@@ -7025,15 +7033,15 @@
         <v>30</v>
       </c>
       <c r="E226" s="3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F226" s="9" t="inlineStr">
         <is>
-          <t>INCOMPLETE</t>
+          <t>FULL (Credit-Exempt)</t>
         </is>
       </c>
       <c r="G226" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="227">
@@ -7085,7 +7093,7 @@
       <c r="E228" s="3" t="n">
         <v>6.5</v>
       </c>
-      <c r="F228" s="9" t="inlineStr">
+      <c r="F228" s="10" t="inlineStr">
         <is>
           <t>INCOMPLETE</t>
         </is>
@@ -7460,15 +7468,15 @@
         <v>30</v>
       </c>
       <c r="E241" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F241" s="8" t="inlineStr">
         <is>
-          <t>INCOMPLETE</t>
+          <t>FULL (Credit-Exempt)</t>
         </is>
       </c>
       <c r="G241" s="5" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="242">
@@ -7721,15 +7729,15 @@
         <v>30</v>
       </c>
       <c r="E250" s="3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F250" s="9" t="inlineStr">
         <is>
-          <t>INCOMPLETE</t>
+          <t>FULL (Credit-Exempt)</t>
         </is>
       </c>
       <c r="G250" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="251">
@@ -8098,15 +8106,15 @@
         <v>30</v>
       </c>
       <c r="E263" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F263" s="8" t="inlineStr">
         <is>
-          <t>INCOMPLETE</t>
+          <t>FULL (Credit-Exempt)</t>
         </is>
       </c>
       <c r="G263" s="5" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="264">
@@ -8419,7 +8427,7 @@
       <c r="E274" s="3" t="n">
         <v>6.5</v>
       </c>
-      <c r="F274" s="9" t="inlineStr">
+      <c r="F274" s="10" t="inlineStr">
         <is>
           <t>INCOMPLETE</t>
         </is>
@@ -9202,7 +9210,7 @@
       <c r="E301" s="6" t="n">
         <v>6.5</v>
       </c>
-      <c r="F301" s="8" t="inlineStr">
+      <c r="F301" s="11" t="inlineStr">
         <is>
           <t>INCOMPLETE</t>
         </is>
@@ -9316,15 +9324,15 @@
         <v>30</v>
       </c>
       <c r="E305" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F305" s="8" t="inlineStr">
         <is>
-          <t>INCOMPLETE</t>
+          <t>FULL (Credit-Exempt)</t>
         </is>
       </c>
       <c r="G305" s="5" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="306">
@@ -11607,15 +11615,15 @@
         <v>30</v>
       </c>
       <c r="E384" s="3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F384" s="9" t="inlineStr">
         <is>
-          <t>INCOMPLETE</t>
+          <t>FULL (Credit-Exempt)</t>
         </is>
       </c>
       <c r="G384" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="385">
@@ -11754,7 +11762,7 @@
       <c r="E389" s="6" t="n">
         <v>6.5</v>
       </c>
-      <c r="F389" s="8" t="inlineStr">
+      <c r="F389" s="11" t="inlineStr">
         <is>
           <t>INCOMPLETE</t>
         </is>
@@ -11812,7 +11820,7 @@
       <c r="E391" s="6" t="n">
         <v>6.5</v>
       </c>
-      <c r="F391" s="8" t="inlineStr">
+      <c r="F391" s="11" t="inlineStr">
         <is>
           <t>INCOMPLETE</t>
         </is>
@@ -11926,15 +11934,15 @@
         <v>30</v>
       </c>
       <c r="E395" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F395" s="8" t="inlineStr">
         <is>
-          <t>INCOMPLETE</t>
+          <t>FULL (Credit-Exempt)</t>
         </is>
       </c>
       <c r="G395" s="5" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="396">
@@ -13173,15 +13181,15 @@
         <v>30</v>
       </c>
       <c r="E438" s="3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F438" s="9" t="inlineStr">
         <is>
-          <t>INCOMPLETE</t>
+          <t>FULL (Credit-Exempt)</t>
         </is>
       </c>
       <c r="G438" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="439">
@@ -13260,15 +13268,15 @@
         <v>30</v>
       </c>
       <c r="E441" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F441" s="8" t="inlineStr">
         <is>
-          <t>INCOMPLETE</t>
+          <t>FULL (Credit-Exempt)</t>
         </is>
       </c>
       <c r="G441" s="5" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="442">
@@ -14623,15 +14631,15 @@
         <v>30</v>
       </c>
       <c r="E488" s="3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F488" s="9" t="inlineStr">
         <is>
-          <t>INCOMPLETE</t>
+          <t>FULL (Credit-Exempt)</t>
         </is>
       </c>
       <c r="G488" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="489">
@@ -14915,7 +14923,7 @@
       <c r="E498" s="3" t="n">
         <v>6.5</v>
       </c>
-      <c r="F498" s="9" t="inlineStr">
+      <c r="F498" s="10" t="inlineStr">
         <is>
           <t>INCOMPLETE</t>
         </is>
@@ -15261,15 +15269,15 @@
         <v>30</v>
       </c>
       <c r="E510" s="3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F510" s="9" t="inlineStr">
         <is>
-          <t>INCOMPLETE</t>
+          <t>FULL (Credit-Exempt)</t>
         </is>
       </c>
       <c r="G510" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="511">
@@ -15321,7 +15329,7 @@
       <c r="E512" s="3" t="n">
         <v>5.5</v>
       </c>
-      <c r="F512" s="9" t="inlineStr">
+      <c r="F512" s="10" t="inlineStr">
         <is>
           <t>INCOMPLETE</t>
         </is>
@@ -15377,15 +15385,15 @@
         <v>30</v>
       </c>
       <c r="E514" s="3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F514" s="9" t="inlineStr">
         <is>
-          <t>INCOMPLETE</t>
+          <t>FULL (Credit-Exempt)</t>
         </is>
       </c>
       <c r="G514" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="515">
@@ -15812,15 +15820,15 @@
         <v>30</v>
       </c>
       <c r="E529" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F529" s="8" t="inlineStr">
         <is>
-          <t>INCOMPLETE</t>
+          <t>FULL (Credit-Exempt)</t>
         </is>
       </c>
       <c r="G529" s="5" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="530">
@@ -15959,7 +15967,7 @@
       <c r="E534" s="3" t="n">
         <v>5.5</v>
       </c>
-      <c r="F534" s="9" t="inlineStr">
+      <c r="F534" s="10" t="inlineStr">
         <is>
           <t>INCOMPLETE</t>
         </is>
@@ -16450,15 +16458,15 @@
         <v>30</v>
       </c>
       <c r="E551" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F551" s="8" t="inlineStr">
         <is>
-          <t>INCOMPLETE</t>
+          <t>FULL (Credit-Exempt)</t>
         </is>
       </c>
       <c r="G551" s="5" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="552">
@@ -16566,15 +16574,15 @@
         <v>30</v>
       </c>
       <c r="E555" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F555" s="8" t="inlineStr">
         <is>
-          <t>INCOMPLETE</t>
+          <t>FULL (Credit-Exempt)</t>
         </is>
       </c>
       <c r="G555" s="5" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="556">
@@ -16682,15 +16690,15 @@
         <v>30</v>
       </c>
       <c r="E559" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F559" s="8" t="inlineStr">
         <is>
-          <t>INCOMPLETE</t>
+          <t>FULL (Credit-Exempt)</t>
         </is>
       </c>
       <c r="G559" s="5" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="560">
@@ -17378,15 +17386,15 @@
         <v>30</v>
       </c>
       <c r="E583" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F583" s="8" t="inlineStr">
         <is>
-          <t>INCOMPLETE</t>
+          <t>FULL (Credit-Exempt)</t>
         </is>
       </c>
       <c r="G583" s="5" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="584">
@@ -17552,15 +17560,15 @@
         <v>30</v>
       </c>
       <c r="E589" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F589" s="8" t="inlineStr">
         <is>
-          <t>INCOMPLETE</t>
+          <t>FULL (Credit-Exempt)</t>
         </is>
       </c>
       <c r="G589" s="5" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="590">
@@ -18047,7 +18055,7 @@
       <c r="E606" s="3" t="n">
         <v>6.5</v>
       </c>
-      <c r="F606" s="9" t="inlineStr">
+      <c r="F606" s="10" t="inlineStr">
         <is>
           <t>INCOMPLETE</t>
         </is>
@@ -18714,7 +18722,7 @@
       <c r="E629" s="6" t="n">
         <v>6.5</v>
       </c>
-      <c r="F629" s="8" t="inlineStr">
+      <c r="F629" s="11" t="inlineStr">
         <is>
           <t>INCOMPLETE</t>
         </is>
@@ -18830,7 +18838,7 @@
       <c r="E633" s="6" t="n">
         <v>6.5</v>
       </c>
-      <c r="F633" s="8" t="inlineStr">
+      <c r="F633" s="11" t="inlineStr">
         <is>
           <t>INCOMPLETE</t>
         </is>
@@ -19002,15 +19010,15 @@
         <v>30</v>
       </c>
       <c r="E639" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F639" s="8" t="inlineStr">
         <is>
-          <t>INCOMPLETE</t>
+          <t>FULL (Credit-Exempt)</t>
         </is>
       </c>
       <c r="G639" s="5" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="640">
@@ -19497,7 +19505,7 @@
       <c r="E656" s="3" t="n">
         <v>6.5</v>
       </c>
-      <c r="F656" s="9" t="inlineStr">
+      <c r="F656" s="10" t="inlineStr">
         <is>
           <t>INCOMPLETE</t>
         </is>
@@ -19553,15 +19561,15 @@
         <v>30</v>
       </c>
       <c r="E658" s="3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F658" s="9" t="inlineStr">
         <is>
-          <t>INCOMPLETE</t>
+          <t>FULL (Credit-Exempt)</t>
         </is>
       </c>
       <c r="G658" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="659">
@@ -19642,7 +19650,7 @@
       <c r="E661" s="6" t="n">
         <v>6.5</v>
       </c>
-      <c r="F661" s="8" t="inlineStr">
+      <c r="F661" s="11" t="inlineStr">
         <is>
           <t>INCOMPLETE</t>
         </is>
@@ -20222,7 +20230,7 @@
       <c r="E681" s="6" t="n">
         <v>6.5</v>
       </c>
-      <c r="F681" s="8" t="inlineStr">
+      <c r="F681" s="11" t="inlineStr">
         <is>
           <t>INCOMPLETE</t>
         </is>
@@ -20568,15 +20576,15 @@
         <v>30</v>
       </c>
       <c r="E693" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F693" s="8" t="inlineStr">
         <is>
-          <t>INCOMPLETE</t>
+          <t>FULL (Credit-Exempt)</t>
         </is>
       </c>
       <c r="G693" s="5" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="694">
@@ -20597,15 +20605,15 @@
         <v>30</v>
       </c>
       <c r="E694" s="3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F694" s="9" t="inlineStr">
         <is>
-          <t>INCOMPLETE</t>
+          <t>FULL (Credit-Exempt)</t>
         </is>
       </c>
       <c r="G694" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="695">
@@ -20628,7 +20636,7 @@
       <c r="E695" s="6" t="n">
         <v>6.5</v>
       </c>
-      <c r="F695" s="8" t="inlineStr">
+      <c r="F695" s="11" t="inlineStr">
         <is>
           <t>INCOMPLETE</t>
         </is>
@@ -20684,15 +20692,15 @@
         <v>30</v>
       </c>
       <c r="E697" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F697" s="8" t="inlineStr">
         <is>
-          <t>INCOMPLETE</t>
+          <t>FULL (Credit-Exempt)</t>
         </is>
       </c>
       <c r="G697" s="5" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="698">
@@ -21005,7 +21013,7 @@
       <c r="E708" s="3" t="n">
         <v>6.5</v>
       </c>
-      <c r="F708" s="9" t="inlineStr">
+      <c r="F708" s="10" t="inlineStr">
         <is>
           <t>INCOMPLETE</t>
         </is>
@@ -21380,15 +21388,15 @@
         <v>30</v>
       </c>
       <c r="E721" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F721" s="8" t="inlineStr">
         <is>
-          <t>INCOMPLETE</t>
+          <t>FULL (Credit-Exempt)</t>
         </is>
       </c>
       <c r="G721" s="5" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="722">
@@ -22107,7 +22115,7 @@
       <c r="E746" s="3" t="n">
         <v>6.5</v>
       </c>
-      <c r="F746" s="9" t="inlineStr">
+      <c r="F746" s="10" t="inlineStr">
         <is>
           <t>INCOMPLETE</t>
         </is>
@@ -22339,7 +22347,7 @@
       <c r="E754" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="F754" s="9" t="inlineStr">
+      <c r="F754" s="10" t="inlineStr">
         <is>
           <t>INCOMPLETE</t>
         </is>
@@ -22743,15 +22751,15 @@
         <v>30</v>
       </c>
       <c r="E768" s="3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F768" s="9" t="inlineStr">
         <is>
-          <t>INCOMPLETE</t>
+          <t>FULL (Credit-Exempt)</t>
         </is>
       </c>
       <c r="G768" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="769">
@@ -23004,15 +23012,15 @@
         <v>30</v>
       </c>
       <c r="E777" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F777" s="8" t="inlineStr">
         <is>
-          <t>INCOMPLETE</t>
+          <t>FULL (Credit-Exempt)</t>
         </is>
       </c>
       <c r="G777" s="5" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="778">
@@ -23412,7 +23420,7 @@
       <c r="E791" s="6" t="n">
         <v>6.5</v>
       </c>
-      <c r="F791" s="8" t="inlineStr">
+      <c r="F791" s="11" t="inlineStr">
         <is>
           <t>INCOMPLETE</t>
         </is>
@@ -23816,15 +23824,15 @@
         <v>30</v>
       </c>
       <c r="E805" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F805" s="8" t="inlineStr">
         <is>
-          <t>INCOMPLETE</t>
+          <t>FULL (Credit-Exempt)</t>
         </is>
       </c>
       <c r="G805" s="5" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>